<commit_message>
Fix missing name fields required by Facebook Ads upload
Added placeholder names (New Campaign, New Ad Set, New Ad) to Campaign Name,
Ad Set Name, and Ad Name columns — Facebook requires either a name or an ID.

https://claude.ai/code/session_01EBpeDmemL9eYP3cAHJxBC6
</commit_message>
<xml_diff>
--- a/template_clean.xlsx
+++ b/template_clean.xlsx
@@ -2707,7 +2707,11 @@
     <row r="2">
       <c r="A2" s="0" t="n"/>
       <c r="B2" s="0" t="n"/>
-      <c r="C2" s="0" t="n"/>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>New Campaign</t>
+        </is>
+      </c>
       <c r="D2" s="0" t="inlineStr"/>
       <c r="E2" s="0" t="inlineStr"/>
       <c r="F2" s="0" t="inlineStr">
@@ -2775,7 +2779,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AA2" s="0" t="n"/>
+      <c r="AA2" s="0" t="inlineStr">
+        <is>
+          <t>New Ad Set</t>
+        </is>
+      </c>
       <c r="AB2" s="0" t="inlineStr">
         <is>
           <t>06/05/2026 11:02:45 am</t>
@@ -3033,7 +3041,11 @@
       </c>
       <c r="FK2" s="0" t="n"/>
       <c r="FL2" s="0" t="n"/>
-      <c r="FM2" s="0" t="n"/>
+      <c r="FM2" s="0" t="inlineStr">
+        <is>
+          <t>New Ad</t>
+        </is>
+      </c>
       <c r="FN2" s="0" t="n"/>
       <c r="FO2" s="0" t="n"/>
       <c r="FP2" s="0" t="n"/>

</xml_diff>